<commit_message>
Update README with detailed instructions for file generation and program updates; modify Excel templates for improved data handling.
</commit_message>
<xml_diff>
--- a/bestilling.xlsx
+++ b/bestilling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/NTNUI-klubbklar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_59F76EE26084DAA0FC28A794295BDA16564F9BAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D53D73E0-C0D2-4902-AF66-313A82CF0016}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_59F76EE26084DAA0FC28A794295BDA16564F9BAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9D2794C-A3EF-4DE8-A657-E60BE047CB7E}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5440" yWindow="5440" windowWidth="2370" windowHeight="560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="340" yWindow="340" windowWidth="2370" windowHeight="560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="15.9.2026" sheetId="2" r:id="rId1"/>
@@ -623,11 +623,11 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -932,20 +932,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J188"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="31.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -980,10 +986,10 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -1008,8 +1014,8 @@
       <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="8"/>
-      <c r="B4" s="7"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1032,8 +1038,8 @@
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="8"/>
-      <c r="B5" s="7"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -1056,8 +1062,8 @@
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="8"/>
-      <c r="B6" s="7"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
@@ -1080,8 +1086,8 @@
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="8"/>
-      <c r="B7" s="7"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
@@ -1104,8 +1110,8 @@
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="8"/>
-      <c r="B8" s="7"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -1128,8 +1134,8 @@
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="8"/>
-      <c r="B9" s="7"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="5"/>
       <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
@@ -1152,8 +1158,8 @@
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="8"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1176,8 +1182,8 @@
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="8"/>
-      <c r="B11" s="7"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="5"/>
       <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1200,8 +1206,8 @@
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="6"/>
+      <c r="B12" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1226,8 +1232,8 @@
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="8"/>
-      <c r="B13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
@@ -1254,8 +1260,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="8"/>
-      <c r="B14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="5"/>
       <c r="C14" s="3" t="s">
         <v>19</v>
       </c>
@@ -1278,8 +1284,8 @@
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="8"/>
-      <c r="B15" s="7"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="5"/>
       <c r="C15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1302,8 +1308,8 @@
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="8"/>
-      <c r="B16" s="7"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="5"/>
       <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
@@ -1330,8 +1336,8 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="8"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="5"/>
       <c r="C17" s="3" t="s">
         <v>22</v>
       </c>
@@ -1358,8 +1364,8 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="8"/>
-      <c r="B18" s="7"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="5"/>
       <c r="C18" s="3" t="s">
         <v>22</v>
       </c>
@@ -1386,8 +1392,8 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="8"/>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="6"/>
+      <c r="B19" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -1412,8 +1418,8 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="8"/>
-      <c r="B20" s="7"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="5"/>
       <c r="C20" s="3" t="s">
         <v>22</v>
       </c>
@@ -1436,8 +1442,8 @@
       <c r="J20" s="3"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="8"/>
-      <c r="B21" s="7"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="5"/>
       <c r="C21" s="3" t="s">
         <v>22</v>
       </c>
@@ -1460,8 +1466,8 @@
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="8"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="6"/>
+      <c r="B22" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -1488,8 +1494,8 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="8"/>
-      <c r="B23" s="7"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="5"/>
       <c r="C23" s="3" t="s">
         <v>19</v>
       </c>
@@ -1512,8 +1518,8 @@
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="8"/>
-      <c r="B24" s="7"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="5"/>
       <c r="C24" s="3" t="s">
         <v>22</v>
       </c>
@@ -1540,8 +1546,8 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="8"/>
-      <c r="B25" s="7"/>
+      <c r="A25" s="6"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="3" t="s">
         <v>22</v>
       </c>
@@ -1568,8 +1574,8 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="8"/>
-      <c r="B26" s="7"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="5"/>
       <c r="C26" s="3" t="s">
         <v>44</v>
       </c>
@@ -1592,8 +1598,8 @@
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="8"/>
-      <c r="B27" s="7" t="s">
+      <c r="A27" s="6"/>
+      <c r="B27" s="5" t="s">
         <v>46</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -1618,8 +1624,8 @@
       <c r="J27" s="3"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="8"/>
-      <c r="B28" s="7"/>
+      <c r="A28" s="6"/>
+      <c r="B28" s="5"/>
       <c r="C28" s="3" t="s">
         <v>47</v>
       </c>
@@ -1644,8 +1650,8 @@
       <c r="J28" s="3"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="8"/>
-      <c r="B29" s="7"/>
+      <c r="A29" s="6"/>
+      <c r="B29" s="5"/>
       <c r="C29" s="3" t="s">
         <v>31</v>
       </c>
@@ -1672,8 +1678,8 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="8"/>
-      <c r="B30" s="7"/>
+      <c r="A30" s="6"/>
+      <c r="B30" s="5"/>
       <c r="C30" s="3" t="s">
         <v>19</v>
       </c>
@@ -1696,8 +1702,8 @@
       <c r="J30" s="3"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="8"/>
-      <c r="B31" s="7"/>
+      <c r="A31" s="6"/>
+      <c r="B31" s="5"/>
       <c r="C31" s="3" t="s">
         <v>19</v>
       </c>
@@ -1720,8 +1726,8 @@
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="8"/>
-      <c r="B32" s="7"/>
+      <c r="A32" s="6"/>
+      <c r="B32" s="5"/>
       <c r="C32" s="3" t="s">
         <v>22</v>
       </c>
@@ -1746,8 +1752,8 @@
       <c r="J32" s="3"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="8"/>
-      <c r="B33" s="7"/>
+      <c r="A33" s="6"/>
+      <c r="B33" s="5"/>
       <c r="C33" s="3" t="s">
         <v>22</v>
       </c>
@@ -1772,8 +1778,8 @@
       <c r="J33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="8"/>
-      <c r="B34" s="7"/>
+      <c r="A34" s="6"/>
+      <c r="B34" s="5"/>
       <c r="C34" s="3" t="s">
         <v>22</v>
       </c>
@@ -1798,8 +1804,8 @@
       <c r="J34" s="3"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="8"/>
-      <c r="B35" s="7" t="s">
+      <c r="A35" s="6"/>
+      <c r="B35" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -1826,8 +1832,8 @@
       <c r="J35" s="3"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A36" s="8"/>
-      <c r="B36" s="7" t="s">
+      <c r="A36" s="6"/>
+      <c r="B36" s="5" t="s">
         <v>54</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -1854,8 +1860,8 @@
       <c r="J36" s="3"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" s="8"/>
-      <c r="B37" s="7"/>
+      <c r="A37" s="6"/>
+      <c r="B37" s="5"/>
       <c r="C37" s="3" t="s">
         <v>19</v>
       </c>
@@ -1878,8 +1884,8 @@
       <c r="J37" s="3"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A38" s="8"/>
-      <c r="B38" s="7"/>
+      <c r="A38" s="6"/>
+      <c r="B38" s="5"/>
       <c r="C38" s="3" t="s">
         <v>19</v>
       </c>
@@ -1902,8 +1908,8 @@
       <c r="J38" s="3"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A39" s="8"/>
-      <c r="B39" s="7"/>
+      <c r="A39" s="6"/>
+      <c r="B39" s="5"/>
       <c r="C39" s="3" t="s">
         <v>22</v>
       </c>
@@ -1926,8 +1932,8 @@
       <c r="J39" s="3"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A40" s="8"/>
-      <c r="B40" s="7"/>
+      <c r="A40" s="6"/>
+      <c r="B40" s="5"/>
       <c r="C40" s="3" t="s">
         <v>44</v>
       </c>
@@ -1950,10 +1956,10 @@
       <c r="J40" s="3"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C41" s="4" t="s">
@@ -1980,8 +1986,8 @@
       <c r="J41" s="4"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A42" s="8"/>
-      <c r="B42" s="5"/>
+      <c r="A42" s="6"/>
+      <c r="B42" s="7"/>
       <c r="C42" s="4" t="s">
         <v>31</v>
       </c>
@@ -2006,8 +2012,8 @@
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A43" s="8"/>
-      <c r="B43" s="5"/>
+      <c r="A43" s="6"/>
+      <c r="B43" s="7"/>
       <c r="C43" s="4" t="s">
         <v>61</v>
       </c>
@@ -2030,8 +2036,8 @@
       <c r="J43" s="4"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="8"/>
-      <c r="B44" s="5"/>
+      <c r="A44" s="6"/>
+      <c r="B44" s="7"/>
       <c r="C44" s="4" t="s">
         <v>61</v>
       </c>
@@ -2054,8 +2060,8 @@
       <c r="J44" s="4"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A45" s="8"/>
-      <c r="B45" s="5"/>
+      <c r="A45" s="6"/>
+      <c r="B45" s="7"/>
       <c r="C45" s="4" t="s">
         <v>61</v>
       </c>
@@ -2078,8 +2084,8 @@
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A46" s="8"/>
-      <c r="B46" s="5"/>
+      <c r="A46" s="6"/>
+      <c r="B46" s="7"/>
       <c r="C46" s="4" t="s">
         <v>13</v>
       </c>
@@ -2104,8 +2110,8 @@
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A47" s="8"/>
-      <c r="B47" s="5"/>
+      <c r="A47" s="6"/>
+      <c r="B47" s="7"/>
       <c r="C47" s="4" t="s">
         <v>13</v>
       </c>
@@ -2130,8 +2136,8 @@
       <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A48" s="8"/>
-      <c r="B48" s="5"/>
+      <c r="A48" s="6"/>
+      <c r="B48" s="7"/>
       <c r="C48" s="4" t="s">
         <v>13</v>
       </c>
@@ -2156,8 +2162,8 @@
       <c r="J48" s="4"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" s="8"/>
-      <c r="B49" s="5"/>
+      <c r="A49" s="6"/>
+      <c r="B49" s="7"/>
       <c r="C49" s="4" t="s">
         <v>19</v>
       </c>
@@ -2180,8 +2186,8 @@
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A50" s="8"/>
-      <c r="B50" s="5"/>
+      <c r="A50" s="6"/>
+      <c r="B50" s="7"/>
       <c r="C50" s="4" t="s">
         <v>19</v>
       </c>
@@ -2204,8 +2210,8 @@
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A51" s="8"/>
-      <c r="B51" s="5"/>
+      <c r="A51" s="6"/>
+      <c r="B51" s="7"/>
       <c r="C51" s="4" t="s">
         <v>22</v>
       </c>
@@ -2230,8 +2236,8 @@
       <c r="J51" s="4"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A52" s="8"/>
-      <c r="B52" s="5"/>
+      <c r="A52" s="6"/>
+      <c r="B52" s="7"/>
       <c r="C52" s="4" t="s">
         <v>22</v>
       </c>
@@ -2256,8 +2262,8 @@
       <c r="J52" s="4"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A53" s="8"/>
-      <c r="B53" s="5"/>
+      <c r="A53" s="6"/>
+      <c r="B53" s="7"/>
       <c r="C53" s="4" t="s">
         <v>22</v>
       </c>
@@ -2282,8 +2288,8 @@
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A54" s="8"/>
-      <c r="B54" s="5"/>
+      <c r="A54" s="6"/>
+      <c r="B54" s="7"/>
       <c r="C54" s="4" t="s">
         <v>22</v>
       </c>
@@ -2308,8 +2314,8 @@
       <c r="J54" s="4"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="8"/>
-      <c r="B55" s="5" t="s">
+      <c r="A55" s="6"/>
+      <c r="B55" s="7" t="s">
         <v>64</v>
       </c>
       <c r="C55" s="4" t="s">
@@ -2334,8 +2340,8 @@
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="8"/>
-      <c r="B56" s="5"/>
+      <c r="A56" s="6"/>
+      <c r="B56" s="7"/>
       <c r="C56" s="4" t="s">
         <v>19</v>
       </c>
@@ -2358,8 +2364,8 @@
       <c r="J56" s="4"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="8"/>
-      <c r="B57" s="5"/>
+      <c r="A57" s="6"/>
+      <c r="B57" s="7"/>
       <c r="C57" s="4" t="s">
         <v>22</v>
       </c>
@@ -2382,8 +2388,8 @@
       <c r="J57" s="4"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A58" s="8"/>
-      <c r="B58" s="5"/>
+      <c r="A58" s="6"/>
+      <c r="B58" s="7"/>
       <c r="C58" s="4" t="s">
         <v>22</v>
       </c>
@@ -2406,8 +2412,8 @@
       <c r="J58" s="4"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A59" s="8"/>
-      <c r="B59" s="5" t="s">
+      <c r="A59" s="6"/>
+      <c r="B59" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C59" s="4" t="s">
@@ -2434,8 +2440,8 @@
       <c r="J59" s="4"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A60" s="8"/>
-      <c r="B60" s="5"/>
+      <c r="A60" s="6"/>
+      <c r="B60" s="7"/>
       <c r="C60" s="4" t="s">
         <v>22</v>
       </c>
@@ -2460,8 +2466,8 @@
       <c r="J60" s="4"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A61" s="8"/>
-      <c r="B61" s="5" t="s">
+      <c r="A61" s="6"/>
+      <c r="B61" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C61" s="4" t="s">
@@ -2486,8 +2492,8 @@
       <c r="J61" s="4"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="8"/>
-      <c r="B62" s="5"/>
+      <c r="A62" s="6"/>
+      <c r="B62" s="7"/>
       <c r="C62" s="4" t="s">
         <v>22</v>
       </c>
@@ -2512,8 +2518,8 @@
       <c r="J62" s="4"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="8"/>
-      <c r="B63" s="5" t="s">
+      <c r="A63" s="6"/>
+      <c r="B63" s="7" t="s">
         <v>69</v>
       </c>
       <c r="C63" s="4" t="s">
@@ -2542,8 +2548,8 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="8"/>
-      <c r="B64" s="5"/>
+      <c r="A64" s="6"/>
+      <c r="B64" s="7"/>
       <c r="C64" s="4" t="s">
         <v>61</v>
       </c>
@@ -2566,8 +2572,8 @@
       <c r="J64" s="4"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" s="8"/>
-      <c r="B65" s="5"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="7"/>
       <c r="C65" s="4" t="s">
         <v>19</v>
       </c>
@@ -2590,8 +2596,8 @@
       <c r="J65" s="4"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="8"/>
-      <c r="B66" s="5"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="7"/>
       <c r="C66" s="4" t="s">
         <v>22</v>
       </c>
@@ -2616,8 +2622,8 @@
       <c r="J66" s="4"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="8"/>
-      <c r="B67" s="5"/>
+      <c r="A67" s="6"/>
+      <c r="B67" s="7"/>
       <c r="C67" s="4" t="s">
         <v>22</v>
       </c>
@@ -2642,8 +2648,8 @@
       <c r="J67" s="4"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A68" s="8"/>
-      <c r="B68" s="5" t="s">
+      <c r="A68" s="6"/>
+      <c r="B68" s="7" t="s">
         <v>71</v>
       </c>
       <c r="C68" s="4" t="s">
@@ -2668,8 +2674,8 @@
       <c r="J68" s="4"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A69" s="8"/>
-      <c r="B69" s="5"/>
+      <c r="A69" s="6"/>
+      <c r="B69" s="7"/>
       <c r="C69" s="4" t="s">
         <v>13</v>
       </c>
@@ -2696,8 +2702,8 @@
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A70" s="8"/>
-      <c r="B70" s="5"/>
+      <c r="A70" s="6"/>
+      <c r="B70" s="7"/>
       <c r="C70" s="4" t="s">
         <v>19</v>
       </c>
@@ -2720,8 +2726,8 @@
       <c r="J70" s="4"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A71" s="8"/>
-      <c r="B71" s="5"/>
+      <c r="A71" s="6"/>
+      <c r="B71" s="7"/>
       <c r="C71" s="4" t="s">
         <v>19</v>
       </c>
@@ -2744,8 +2750,8 @@
       <c r="J71" s="4"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A72" s="8"/>
-      <c r="B72" s="5"/>
+      <c r="A72" s="6"/>
+      <c r="B72" s="7"/>
       <c r="C72" s="4" t="s">
         <v>22</v>
       </c>
@@ -2772,8 +2778,8 @@
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A73" s="8"/>
-      <c r="B73" s="5"/>
+      <c r="A73" s="6"/>
+      <c r="B73" s="7"/>
       <c r="C73" s="4" t="s">
         <v>22</v>
       </c>
@@ -2800,8 +2806,8 @@
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A74" s="8"/>
-      <c r="B74" s="5"/>
+      <c r="A74" s="6"/>
+      <c r="B74" s="7"/>
       <c r="C74" s="4" t="s">
         <v>22</v>
       </c>
@@ -2828,8 +2834,8 @@
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A75" s="8"/>
-      <c r="B75" s="5"/>
+      <c r="A75" s="6"/>
+      <c r="B75" s="7"/>
       <c r="C75" s="4" t="s">
         <v>22</v>
       </c>
@@ -2856,10 +2862,10 @@
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B76" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C76" s="3" t="s">
@@ -2884,8 +2890,8 @@
       <c r="J76" s="3"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A77" s="8"/>
-      <c r="B77" s="7"/>
+      <c r="A77" s="6"/>
+      <c r="B77" s="5"/>
       <c r="C77" s="3" t="s">
         <v>19</v>
       </c>
@@ -2908,8 +2914,8 @@
       <c r="J77" s="3"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A78" s="8"/>
-      <c r="B78" s="7"/>
+      <c r="A78" s="6"/>
+      <c r="B78" s="5"/>
       <c r="C78" s="3" t="s">
         <v>19</v>
       </c>
@@ -2932,8 +2938,8 @@
       <c r="J78" s="3"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A79" s="8"/>
-      <c r="B79" s="7"/>
+      <c r="A79" s="6"/>
+      <c r="B79" s="5"/>
       <c r="C79" s="3" t="s">
         <v>22</v>
       </c>
@@ -2956,8 +2962,8 @@
       <c r="J79" s="3"/>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A80" s="8"/>
-      <c r="B80" s="7" t="s">
+      <c r="A80" s="6"/>
+      <c r="B80" s="5" t="s">
         <v>77</v>
       </c>
       <c r="C80" s="3" t="s">
@@ -2984,8 +2990,8 @@
       <c r="J80" s="3"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A81" s="8"/>
-      <c r="B81" s="7"/>
+      <c r="A81" s="6"/>
+      <c r="B81" s="5"/>
       <c r="C81" s="3" t="s">
         <v>79</v>
       </c>
@@ -3008,8 +3014,8 @@
       <c r="J81" s="3"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A82" s="8"/>
-      <c r="B82" s="7"/>
+      <c r="A82" s="6"/>
+      <c r="B82" s="5"/>
       <c r="C82" s="3" t="s">
         <v>19</v>
       </c>
@@ -3032,8 +3038,8 @@
       <c r="J82" s="3"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A83" s="8"/>
-      <c r="B83" s="7"/>
+      <c r="A83" s="6"/>
+      <c r="B83" s="5"/>
       <c r="C83" s="3" t="s">
         <v>22</v>
       </c>
@@ -3058,8 +3064,8 @@
       <c r="J83" s="3"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A84" s="8"/>
-      <c r="B84" s="7"/>
+      <c r="A84" s="6"/>
+      <c r="B84" s="5"/>
       <c r="C84" s="3" t="s">
         <v>22</v>
       </c>
@@ -3084,8 +3090,8 @@
       <c r="J84" s="3"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A85" s="8"/>
-      <c r="B85" s="7" t="s">
+      <c r="A85" s="6"/>
+      <c r="B85" s="5" t="s">
         <v>81</v>
       </c>
       <c r="C85" s="3" t="s">
@@ -3110,8 +3116,8 @@
       <c r="J85" s="3"/>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A86" s="8"/>
-      <c r="B86" s="7"/>
+      <c r="A86" s="6"/>
+      <c r="B86" s="5"/>
       <c r="C86" s="3" t="s">
         <v>19</v>
       </c>
@@ -3134,8 +3140,8 @@
       <c r="J86" s="3"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A87" s="8"/>
-      <c r="B87" s="7"/>
+      <c r="A87" s="6"/>
+      <c r="B87" s="5"/>
       <c r="C87" s="3" t="s">
         <v>22</v>
       </c>
@@ -3161,7 +3167,7 @@
       <c r="A88" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="7" t="s">
         <v>83</v>
       </c>
       <c r="C88" s="4" t="s">
@@ -3190,10 +3196,10 @@
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A89" s="8" t="s">
+      <c r="A89" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="B89" s="5" t="s">
         <v>87</v>
       </c>
       <c r="C89" s="3" t="s">
@@ -3220,8 +3226,8 @@
       <c r="J89" s="3"/>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A90" s="8"/>
-      <c r="B90" s="7"/>
+      <c r="A90" s="6"/>
+      <c r="B90" s="5"/>
       <c r="C90" s="3" t="s">
         <v>19</v>
       </c>
@@ -3244,8 +3250,8 @@
       <c r="J90" s="3"/>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A91" s="8"/>
-      <c r="B91" s="7"/>
+      <c r="A91" s="6"/>
+      <c r="B91" s="5"/>
       <c r="C91" s="3" t="s">
         <v>19</v>
       </c>
@@ -3268,8 +3274,8 @@
       <c r="J91" s="3"/>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A92" s="8"/>
-      <c r="B92" s="7"/>
+      <c r="A92" s="6"/>
+      <c r="B92" s="5"/>
       <c r="C92" s="3" t="s">
         <v>22</v>
       </c>
@@ -3294,8 +3300,8 @@
       <c r="J92" s="3"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A93" s="8"/>
-      <c r="B93" s="7" t="s">
+      <c r="A93" s="6"/>
+      <c r="B93" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C93" s="3" t="s">
@@ -3322,8 +3328,8 @@
       <c r="J93" s="3"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A94" s="8"/>
-      <c r="B94" s="7"/>
+      <c r="A94" s="6"/>
+      <c r="B94" s="5"/>
       <c r="C94" s="3" t="s">
         <v>19</v>
       </c>
@@ -3346,8 +3352,8 @@
       <c r="J94" s="3"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A95" s="8"/>
-      <c r="B95" s="7"/>
+      <c r="A95" s="6"/>
+      <c r="B95" s="5"/>
       <c r="C95" s="3" t="s">
         <v>22</v>
       </c>
@@ -3372,8 +3378,8 @@
       <c r="J95" s="3"/>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A96" s="8"/>
-      <c r="B96" s="7"/>
+      <c r="A96" s="6"/>
+      <c r="B96" s="5"/>
       <c r="C96" s="3" t="s">
         <v>22</v>
       </c>
@@ -3398,8 +3404,8 @@
       <c r="J96" s="3"/>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A97" s="8"/>
-      <c r="B97" s="7"/>
+      <c r="A97" s="6"/>
+      <c r="B97" s="5"/>
       <c r="C97" s="3" t="s">
         <v>22</v>
       </c>
@@ -3424,8 +3430,8 @@
       <c r="J97" s="3"/>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A98" s="8"/>
-      <c r="B98" s="7" t="s">
+      <c r="A98" s="6"/>
+      <c r="B98" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C98" s="3" t="s">
@@ -3452,8 +3458,8 @@
       <c r="J98" s="3"/>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A99" s="8"/>
-      <c r="B99" s="7"/>
+      <c r="A99" s="6"/>
+      <c r="B99" s="5"/>
       <c r="C99" s="3" t="s">
         <v>61</v>
       </c>
@@ -3476,8 +3482,8 @@
       <c r="J99" s="3"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A100" s="8"/>
-      <c r="B100" s="7"/>
+      <c r="A100" s="6"/>
+      <c r="B100" s="5"/>
       <c r="C100" s="3" t="s">
         <v>22</v>
       </c>
@@ -3502,8 +3508,8 @@
       <c r="J100" s="3"/>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A101" s="8"/>
-      <c r="B101" s="7" t="s">
+      <c r="A101" s="6"/>
+      <c r="B101" s="5" t="s">
         <v>93</v>
       </c>
       <c r="C101" s="3" t="s">
@@ -3530,8 +3536,8 @@
       <c r="J101" s="3"/>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A102" s="8"/>
-      <c r="B102" s="7"/>
+      <c r="A102" s="6"/>
+      <c r="B102" s="5"/>
       <c r="C102" s="3" t="s">
         <v>95</v>
       </c>
@@ -3550,8 +3556,8 @@
       <c r="J102" s="3"/>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A103" s="8"/>
-      <c r="B103" s="7"/>
+      <c r="A103" s="6"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="3" t="s">
         <v>95</v>
       </c>
@@ -3570,10 +3576,10 @@
       <c r="J103" s="3"/>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A104" s="8" t="s">
+      <c r="A104" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B104" s="7" t="s">
         <v>98</v>
       </c>
       <c r="C104" s="4" t="s">
@@ -3600,8 +3606,8 @@
       <c r="J104" s="4"/>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A105" s="8"/>
-      <c r="B105" s="5"/>
+      <c r="A105" s="6"/>
+      <c r="B105" s="7"/>
       <c r="C105" s="4" t="s">
         <v>61</v>
       </c>
@@ -3624,8 +3630,8 @@
       <c r="J105" s="4"/>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A106" s="8"/>
-      <c r="B106" s="5"/>
+      <c r="A106" s="6"/>
+      <c r="B106" s="7"/>
       <c r="C106" s="4" t="s">
         <v>100</v>
       </c>
@@ -3650,10 +3656,10 @@
       <c r="J106" s="4"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A107" s="8" t="s">
+      <c r="A107" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B107" s="7" t="s">
+      <c r="B107" s="5" t="s">
         <v>103</v>
       </c>
       <c r="C107" s="3" t="s">
@@ -3680,8 +3686,8 @@
       <c r="J107" s="3"/>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A108" s="8"/>
-      <c r="B108" s="7"/>
+      <c r="A108" s="6"/>
+      <c r="B108" s="5"/>
       <c r="C108" s="3" t="s">
         <v>47</v>
       </c>
@@ -3706,8 +3712,8 @@
       <c r="J108" s="3"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A109" s="8"/>
-      <c r="B109" s="7"/>
+      <c r="A109" s="6"/>
+      <c r="B109" s="5"/>
       <c r="C109" s="3" t="s">
         <v>61</v>
       </c>
@@ -3730,8 +3736,8 @@
       <c r="J109" s="3"/>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A110" s="8"/>
-      <c r="B110" s="7"/>
+      <c r="A110" s="6"/>
+      <c r="B110" s="5"/>
       <c r="C110" s="3" t="s">
         <v>19</v>
       </c>
@@ -3754,8 +3760,8 @@
       <c r="J110" s="3"/>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A111" s="8"/>
-      <c r="B111" s="7"/>
+      <c r="A111" s="6"/>
+      <c r="B111" s="5"/>
       <c r="C111" s="3" t="s">
         <v>22</v>
       </c>
@@ -3780,8 +3786,8 @@
       <c r="J111" s="3"/>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A112" s="8"/>
-      <c r="B112" s="7"/>
+      <c r="A112" s="6"/>
+      <c r="B112" s="5"/>
       <c r="C112" s="3" t="s">
         <v>22</v>
       </c>
@@ -3806,8 +3812,8 @@
       <c r="J112" s="3"/>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A113" s="8"/>
-      <c r="B113" s="7"/>
+      <c r="A113" s="6"/>
+      <c r="B113" s="5"/>
       <c r="C113" s="3" t="s">
         <v>22</v>
       </c>
@@ -3832,8 +3838,8 @@
       <c r="J113" s="3"/>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A114" s="8"/>
-      <c r="B114" s="7" t="s">
+      <c r="A114" s="6"/>
+      <c r="B114" s="5" t="s">
         <v>105</v>
       </c>
       <c r="C114" s="3" t="s">
@@ -3858,8 +3864,8 @@
       <c r="J114" s="3"/>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A115" s="8"/>
-      <c r="B115" s="7"/>
+      <c r="A115" s="6"/>
+      <c r="B115" s="5"/>
       <c r="C115" s="3" t="s">
         <v>22</v>
       </c>
@@ -3884,8 +3890,8 @@
       <c r="J115" s="3"/>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A116" s="8"/>
-      <c r="B116" s="7" t="s">
+      <c r="A116" s="6"/>
+      <c r="B116" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C116" s="3" t="s">
@@ -3912,8 +3918,8 @@
       <c r="J116" s="3"/>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A117" s="8"/>
-      <c r="B117" s="7"/>
+      <c r="A117" s="6"/>
+      <c r="B117" s="5"/>
       <c r="C117" s="3" t="s">
         <v>19</v>
       </c>
@@ -3936,8 +3942,8 @@
       <c r="J117" s="3"/>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A118" s="8"/>
-      <c r="B118" s="7"/>
+      <c r="A118" s="6"/>
+      <c r="B118" s="5"/>
       <c r="C118" s="3" t="s">
         <v>22</v>
       </c>
@@ -3964,10 +3970,10 @@
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A119" s="8" t="s">
+      <c r="A119" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B119" s="5" t="s">
+      <c r="B119" s="7" t="s">
         <v>111</v>
       </c>
       <c r="C119" s="4" t="s">
@@ -3992,8 +3998,8 @@
       <c r="J119" s="4"/>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A120" s="8"/>
-      <c r="B120" s="5"/>
+      <c r="A120" s="6"/>
+      <c r="B120" s="7"/>
       <c r="C120" s="4" t="s">
         <v>112</v>
       </c>
@@ -4016,8 +4022,8 @@
       <c r="J120" s="4"/>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A121" s="8"/>
-      <c r="B121" s="5"/>
+      <c r="A121" s="6"/>
+      <c r="B121" s="7"/>
       <c r="C121" s="4" t="s">
         <v>112</v>
       </c>
@@ -4040,8 +4046,8 @@
       <c r="J121" s="4"/>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A122" s="8"/>
-      <c r="B122" s="5" t="s">
+      <c r="A122" s="6"/>
+      <c r="B122" s="7" t="s">
         <v>114</v>
       </c>
       <c r="C122" s="4" t="s">
@@ -4070,8 +4076,8 @@
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A123" s="8"/>
-      <c r="B123" s="5"/>
+      <c r="A123" s="6"/>
+      <c r="B123" s="7"/>
       <c r="C123" s="4" t="s">
         <v>61</v>
       </c>
@@ -4094,8 +4100,8 @@
       <c r="J123" s="4"/>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A124" s="8"/>
-      <c r="B124" s="5"/>
+      <c r="A124" s="6"/>
+      <c r="B124" s="7"/>
       <c r="C124" s="4" t="s">
         <v>112</v>
       </c>
@@ -4120,8 +4126,8 @@
       <c r="J124" s="4"/>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A125" s="8"/>
-      <c r="B125" s="5"/>
+      <c r="A125" s="6"/>
+      <c r="B125" s="7"/>
       <c r="C125" s="4" t="s">
         <v>112</v>
       </c>
@@ -4146,8 +4152,8 @@
       <c r="J125" s="4"/>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A126" s="8"/>
-      <c r="B126" s="5" t="s">
+      <c r="A126" s="6"/>
+      <c r="B126" s="7" t="s">
         <v>118</v>
       </c>
       <c r="C126" s="4" t="s">
@@ -4172,8 +4178,8 @@
       <c r="J126" s="4"/>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A127" s="8"/>
-      <c r="B127" s="5"/>
+      <c r="A127" s="6"/>
+      <c r="B127" s="7"/>
       <c r="C127" s="4" t="s">
         <v>112</v>
       </c>
@@ -4196,8 +4202,8 @@
       <c r="J127" s="4"/>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A128" s="8"/>
-      <c r="B128" s="5" t="s">
+      <c r="A128" s="6"/>
+      <c r="B128" s="7" t="s">
         <v>119</v>
       </c>
       <c r="C128" s="4" t="s">
@@ -4224,8 +4230,8 @@
       <c r="J128" s="4"/>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A129" s="8"/>
-      <c r="B129" s="5"/>
+      <c r="A129" s="6"/>
+      <c r="B129" s="7"/>
       <c r="C129" s="4" t="s">
         <v>100</v>
       </c>
@@ -4250,8 +4256,8 @@
       <c r="J129" s="4"/>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A130" s="8"/>
-      <c r="B130" s="5"/>
+      <c r="A130" s="6"/>
+      <c r="B130" s="7"/>
       <c r="C130" s="4" t="s">
         <v>112</v>
       </c>
@@ -4274,8 +4280,8 @@
       <c r="J130" s="4"/>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A131" s="8"/>
-      <c r="B131" s="5" t="s">
+      <c r="A131" s="6"/>
+      <c r="B131" s="7" t="s">
         <v>121</v>
       </c>
       <c r="C131" s="4" t="s">
@@ -4304,8 +4310,8 @@
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A132" s="8"/>
-      <c r="B132" s="5"/>
+      <c r="A132" s="6"/>
+      <c r="B132" s="7"/>
       <c r="C132" s="4" t="s">
         <v>100</v>
       </c>
@@ -4332,8 +4338,8 @@
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A133" s="8"/>
-      <c r="B133" s="5"/>
+      <c r="A133" s="6"/>
+      <c r="B133" s="7"/>
       <c r="C133" s="4" t="s">
         <v>112</v>
       </c>
@@ -4360,8 +4366,8 @@
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A134" s="8"/>
-      <c r="B134" s="5"/>
+      <c r="A134" s="6"/>
+      <c r="B134" s="7"/>
       <c r="C134" s="4" t="s">
         <v>112</v>
       </c>
@@ -4388,8 +4394,8 @@
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A135" s="8"/>
-      <c r="B135" s="5"/>
+      <c r="A135" s="6"/>
+      <c r="B135" s="7"/>
       <c r="C135" s="4" t="s">
         <v>112</v>
       </c>
@@ -4416,8 +4422,8 @@
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A136" s="8"/>
-      <c r="B136" s="5" t="s">
+      <c r="A136" s="6"/>
+      <c r="B136" s="7" t="s">
         <v>124</v>
       </c>
       <c r="C136" s="4" t="s">
@@ -4444,8 +4450,8 @@
       <c r="J136" s="4"/>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A137" s="8"/>
-      <c r="B137" s="5"/>
+      <c r="A137" s="6"/>
+      <c r="B137" s="7"/>
       <c r="C137" s="4" t="s">
         <v>112</v>
       </c>
@@ -4470,8 +4476,8 @@
       <c r="J137" s="4"/>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A138" s="8"/>
-      <c r="B138" s="5" t="s">
+      <c r="A138" s="6"/>
+      <c r="B138" s="7" t="s">
         <v>126</v>
       </c>
       <c r="C138" s="4" t="s">
@@ -4496,8 +4502,8 @@
       <c r="J138" s="4"/>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A139" s="8"/>
-      <c r="B139" s="5"/>
+      <c r="A139" s="6"/>
+      <c r="B139" s="7"/>
       <c r="C139" s="4" t="s">
         <v>112</v>
       </c>
@@ -4520,8 +4526,8 @@
       <c r="J139" s="4"/>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A140" s="8"/>
-      <c r="B140" s="5"/>
+      <c r="A140" s="6"/>
+      <c r="B140" s="7"/>
       <c r="C140" s="4" t="s">
         <v>112</v>
       </c>
@@ -4544,8 +4550,8 @@
       <c r="J140" s="4"/>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A141" s="8"/>
-      <c r="B141" s="5"/>
+      <c r="A141" s="6"/>
+      <c r="B141" s="7"/>
       <c r="C141" s="4" t="s">
         <v>112</v>
       </c>
@@ -4568,10 +4574,10 @@
       <c r="J141" s="4"/>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A142" s="8" t="s">
+      <c r="A142" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B142" s="7" t="s">
+      <c r="B142" s="5" t="s">
         <v>128</v>
       </c>
       <c r="C142" s="3" t="s">
@@ -4598,8 +4604,8 @@
       <c r="J142" s="3"/>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A143" s="8"/>
-      <c r="B143" s="7"/>
+      <c r="A143" s="6"/>
+      <c r="B143" s="5"/>
       <c r="C143" s="3" t="s">
         <v>100</v>
       </c>
@@ -4624,8 +4630,8 @@
       <c r="J143" s="3"/>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A144" s="8"/>
-      <c r="B144" s="7"/>
+      <c r="A144" s="6"/>
+      <c r="B144" s="5"/>
       <c r="C144" s="3" t="s">
         <v>112</v>
       </c>
@@ -4650,8 +4656,8 @@
       <c r="J144" s="3"/>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A145" s="8"/>
-      <c r="B145" s="7"/>
+      <c r="A145" s="6"/>
+      <c r="B145" s="5"/>
       <c r="C145" s="3" t="s">
         <v>112</v>
       </c>
@@ -4676,8 +4682,8 @@
       <c r="J145" s="3"/>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A146" s="8"/>
-      <c r="B146" s="7" t="s">
+      <c r="A146" s="6"/>
+      <c r="B146" s="5" t="s">
         <v>130</v>
       </c>
       <c r="C146" s="3" t="s">
@@ -4704,8 +4710,8 @@
       <c r="J146" s="3"/>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A147" s="8"/>
-      <c r="B147" s="7"/>
+      <c r="A147" s="6"/>
+      <c r="B147" s="5"/>
       <c r="C147" s="3" t="s">
         <v>61</v>
       </c>
@@ -4728,8 +4734,8 @@
       <c r="J147" s="3"/>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A148" s="8"/>
-      <c r="B148" s="7"/>
+      <c r="A148" s="6"/>
+      <c r="B148" s="5"/>
       <c r="C148" s="3" t="s">
         <v>100</v>
       </c>
@@ -4754,8 +4760,8 @@
       <c r="J148" s="3"/>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A149" s="8"/>
-      <c r="B149" s="7"/>
+      <c r="A149" s="6"/>
+      <c r="B149" s="5"/>
       <c r="C149" s="3" t="s">
         <v>112</v>
       </c>
@@ -4780,8 +4786,8 @@
       <c r="J149" s="3"/>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A150" s="8"/>
-      <c r="B150" s="7"/>
+      <c r="A150" s="6"/>
+      <c r="B150" s="5"/>
       <c r="C150" s="3" t="s">
         <v>112</v>
       </c>
@@ -4806,8 +4812,8 @@
       <c r="J150" s="3"/>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A151" s="8"/>
-      <c r="B151" s="7" t="s">
+      <c r="A151" s="6"/>
+      <c r="B151" s="5" t="s">
         <v>135</v>
       </c>
       <c r="C151" s="3" t="s">
@@ -4834,8 +4840,8 @@
       <c r="J151" s="3"/>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A152" s="8"/>
-      <c r="B152" s="7"/>
+      <c r="A152" s="6"/>
+      <c r="B152" s="5"/>
       <c r="C152" s="3" t="s">
         <v>100</v>
       </c>
@@ -4860,8 +4866,8 @@
       <c r="J152" s="3"/>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A153" s="8"/>
-      <c r="B153" s="7"/>
+      <c r="A153" s="6"/>
+      <c r="B153" s="5"/>
       <c r="C153" s="3" t="s">
         <v>112</v>
       </c>
@@ -4886,8 +4892,8 @@
       <c r="J153" s="3"/>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A154" s="8"/>
-      <c r="B154" s="7"/>
+      <c r="A154" s="6"/>
+      <c r="B154" s="5"/>
       <c r="C154" s="3" t="s">
         <v>112</v>
       </c>
@@ -4912,10 +4918,10 @@
       <c r="J154" s="3"/>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A155" s="8" t="s">
+      <c r="A155" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B155" s="5" t="s">
+      <c r="B155" s="7" t="s">
         <v>138</v>
       </c>
       <c r="C155" s="4" t="s">
@@ -4940,8 +4946,8 @@
       <c r="J155" s="4"/>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A156" s="8"/>
-      <c r="B156" s="5"/>
+      <c r="A156" s="6"/>
+      <c r="B156" s="7"/>
       <c r="C156" s="4" t="s">
         <v>112</v>
       </c>
@@ -4966,10 +4972,10 @@
       <c r="J156" s="4"/>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A157" s="8" t="s">
+      <c r="A157" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B157" s="7" t="s">
+      <c r="B157" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C157" s="3" t="s">
@@ -4996,8 +5002,8 @@
       <c r="J157" s="3"/>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A158" s="8"/>
-      <c r="B158" s="7"/>
+      <c r="A158" s="6"/>
+      <c r="B158" s="5"/>
       <c r="C158" s="3" t="s">
         <v>115</v>
       </c>
@@ -5024,8 +5030,8 @@
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A159" s="8"/>
-      <c r="B159" s="7"/>
+      <c r="A159" s="6"/>
+      <c r="B159" s="5"/>
       <c r="C159" s="3" t="s">
         <v>100</v>
       </c>
@@ -5050,8 +5056,8 @@
       <c r="J159" s="3"/>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A160" s="8"/>
-      <c r="B160" s="7"/>
+      <c r="A160" s="6"/>
+      <c r="B160" s="5"/>
       <c r="C160" s="3" t="s">
         <v>112</v>
       </c>
@@ -5074,8 +5080,8 @@
       <c r="J160" s="3"/>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A161" s="8"/>
-      <c r="B161" s="7"/>
+      <c r="A161" s="6"/>
+      <c r="B161" s="5"/>
       <c r="C161" s="3" t="s">
         <v>112</v>
       </c>
@@ -5098,8 +5104,8 @@
       <c r="J161" s="3"/>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A162" s="8"/>
-      <c r="B162" s="7"/>
+      <c r="A162" s="6"/>
+      <c r="B162" s="5"/>
       <c r="C162" s="3" t="s">
         <v>112</v>
       </c>
@@ -5122,8 +5128,8 @@
       <c r="J162" s="3"/>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A163" s="8"/>
-      <c r="B163" s="7"/>
+      <c r="A163" s="6"/>
+      <c r="B163" s="5"/>
       <c r="C163" s="3" t="s">
         <v>44</v>
       </c>
@@ -5146,10 +5152,10 @@
       <c r="J163" s="3"/>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A164" s="8" t="s">
+      <c r="A164" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B164" s="5" t="s">
+      <c r="B164" s="7" t="s">
         <v>147</v>
       </c>
       <c r="C164" s="4" t="s">
@@ -5176,8 +5182,8 @@
       <c r="J164" s="4"/>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A165" s="8"/>
-      <c r="B165" s="5"/>
+      <c r="A165" s="6"/>
+      <c r="B165" s="7"/>
       <c r="C165" s="4" t="s">
         <v>112</v>
       </c>
@@ -5202,10 +5208,10 @@
       <c r="J165" s="4"/>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A166" s="8" t="s">
+      <c r="A166" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B166" s="7" t="s">
+      <c r="B166" s="5" t="s">
         <v>150</v>
       </c>
       <c r="C166" s="3" t="s">
@@ -5232,8 +5238,8 @@
       <c r="J166" s="3"/>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A167" s="8"/>
-      <c r="B167" s="7"/>
+      <c r="A167" s="6"/>
+      <c r="B167" s="5"/>
       <c r="C167" s="3" t="s">
         <v>112</v>
       </c>
@@ -5258,8 +5264,8 @@
       <c r="J167" s="3"/>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A168" s="8"/>
-      <c r="B168" s="7"/>
+      <c r="A168" s="6"/>
+      <c r="B168" s="5"/>
       <c r="C168" s="3" t="s">
         <v>112</v>
       </c>
@@ -5284,8 +5290,8 @@
       <c r="J168" s="3"/>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A169" s="8"/>
-      <c r="B169" s="7" t="s">
+      <c r="A169" s="6"/>
+      <c r="B169" s="5" t="s">
         <v>152</v>
       </c>
       <c r="C169" s="3" t="s">
@@ -5312,8 +5318,8 @@
       <c r="J169" s="3"/>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A170" s="8"/>
-      <c r="B170" s="7"/>
+      <c r="A170" s="6"/>
+      <c r="B170" s="5"/>
       <c r="C170" s="3" t="s">
         <v>112</v>
       </c>
@@ -5338,8 +5344,8 @@
       <c r="J170" s="3"/>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A171" s="8"/>
-      <c r="B171" s="7" t="s">
+      <c r="A171" s="6"/>
+      <c r="B171" s="5" t="s">
         <v>156</v>
       </c>
       <c r="C171" s="3" t="s">
@@ -5364,10 +5370,10 @@
       <c r="J171" s="3"/>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A172" s="8" t="s">
+      <c r="A172" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B172" s="5" t="s">
+      <c r="B172" s="7" t="s">
         <v>158</v>
       </c>
       <c r="C172" s="4" t="s">
@@ -5394,8 +5400,8 @@
       <c r="J172" s="4"/>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A173" s="8"/>
-      <c r="B173" s="5" t="s">
+      <c r="A173" s="6"/>
+      <c r="B173" s="7" t="s">
         <v>160</v>
       </c>
       <c r="C173" s="4" t="s">
@@ -5422,8 +5428,8 @@
       <c r="J173" s="4"/>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A174" s="8"/>
-      <c r="B174" s="5" t="s">
+      <c r="A174" s="6"/>
+      <c r="B174" s="7" t="s">
         <v>162</v>
       </c>
       <c r="C174" s="4" t="s">
@@ -5448,8 +5454,8 @@
       <c r="J174" s="4"/>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A175" s="8"/>
-      <c r="B175" s="5"/>
+      <c r="A175" s="6"/>
+      <c r="B175" s="7"/>
       <c r="C175" s="4" t="s">
         <v>163</v>
       </c>
@@ -5472,8 +5478,8 @@
       <c r="J175" s="4"/>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A176" s="8"/>
-      <c r="B176" s="5"/>
+      <c r="A176" s="6"/>
+      <c r="B176" s="7"/>
       <c r="C176" s="4" t="s">
         <v>95</v>
       </c>
@@ -5492,8 +5498,8 @@
       <c r="J176" s="4"/>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A177" s="8"/>
-      <c r="B177" s="5"/>
+      <c r="A177" s="6"/>
+      <c r="B177" s="7"/>
       <c r="C177" s="4" t="s">
         <v>112</v>
       </c>
@@ -5518,8 +5524,8 @@
       <c r="J177" s="4"/>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A178" s="8"/>
-      <c r="B178" s="5"/>
+      <c r="A178" s="6"/>
+      <c r="B178" s="7"/>
       <c r="C178" s="4" t="s">
         <v>112</v>
       </c>
@@ -5544,8 +5550,8 @@
       <c r="J178" s="4"/>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A179" s="8"/>
-      <c r="B179" s="5"/>
+      <c r="A179" s="6"/>
+      <c r="B179" s="7"/>
       <c r="C179" s="4" t="s">
         <v>112</v>
       </c>
@@ -5570,8 +5576,8 @@
       <c r="J179" s="4"/>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A180" s="8"/>
-      <c r="B180" s="5" t="s">
+      <c r="A180" s="6"/>
+      <c r="B180" s="7" t="s">
         <v>166</v>
       </c>
       <c r="C180" s="4" t="s">
@@ -5596,8 +5602,8 @@
       <c r="J180" s="4"/>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A181" s="8"/>
-      <c r="B181" s="5"/>
+      <c r="A181" s="6"/>
+      <c r="B181" s="7"/>
       <c r="C181" s="4" t="s">
         <v>163</v>
       </c>
@@ -5620,8 +5626,8 @@
       <c r="J181" s="4"/>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A182" s="8"/>
-      <c r="B182" s="5"/>
+      <c r="A182" s="6"/>
+      <c r="B182" s="7"/>
       <c r="C182" s="4" t="s">
         <v>112</v>
       </c>
@@ -5644,8 +5650,8 @@
       <c r="J182" s="4"/>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A183" s="8"/>
-      <c r="B183" s="5" t="s">
+      <c r="A183" s="6"/>
+      <c r="B183" s="7" t="s">
         <v>167</v>
       </c>
       <c r="C183" s="4" t="s">
@@ -5674,8 +5680,8 @@
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A184" s="8"/>
-      <c r="B184" s="5"/>
+      <c r="A184" s="6"/>
+      <c r="B184" s="7"/>
       <c r="C184" s="4" t="s">
         <v>112</v>
       </c>
@@ -5702,10 +5708,10 @@
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A185" s="8" t="s">
+      <c r="A185" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B185" s="7" t="s">
+      <c r="B185" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C185" s="3" t="s">
@@ -5732,8 +5738,8 @@
       <c r="J185" s="3"/>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A186" s="8"/>
-      <c r="B186" s="7"/>
+      <c r="A186" s="6"/>
+      <c r="B186" s="5"/>
       <c r="C186" s="3" t="s">
         <v>100</v>
       </c>
@@ -5758,8 +5764,8 @@
       <c r="J186" s="3"/>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A187" s="8"/>
-      <c r="B187" s="7"/>
+      <c r="A187" s="6"/>
+      <c r="B187" s="5"/>
       <c r="C187" s="3" t="s">
         <v>112</v>
       </c>
@@ -5782,8 +5788,8 @@
       <c r="J187" s="3"/>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A188" s="8"/>
-      <c r="B188" s="7"/>
+      <c r="A188" s="6"/>
+      <c r="B188" s="5"/>
       <c r="C188" s="3" t="s">
         <v>112</v>
       </c>
@@ -5807,26 +5813,20 @@
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="A142:A154"/>
-    <mergeCell ref="B119:B121"/>
-    <mergeCell ref="A185:A188"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B164:B165"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="B185:B188"/>
-    <mergeCell ref="B93:B97"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="A155:A156"/>
-    <mergeCell ref="B114:B115"/>
-    <mergeCell ref="B116:B118"/>
-    <mergeCell ref="A157:A163"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="A76:A87"/>
-    <mergeCell ref="B88"/>
-    <mergeCell ref="B27:B34"/>
+    <mergeCell ref="B172"/>
+    <mergeCell ref="A3:A40"/>
+    <mergeCell ref="B76:B79"/>
+    <mergeCell ref="A166:A171"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="B107:B113"/>
+    <mergeCell ref="A172:A184"/>
+    <mergeCell ref="B146:B150"/>
+    <mergeCell ref="B183:B184"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="B157:B163"/>
+    <mergeCell ref="B136:B137"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A119:A141"/>
     <mergeCell ref="B131:B135"/>
@@ -5843,11 +5843,31 @@
     <mergeCell ref="A104:A106"/>
     <mergeCell ref="B138:B141"/>
     <mergeCell ref="B35"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B164:B165"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="B185:B188"/>
+    <mergeCell ref="B93:B97"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="B116:B118"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="B88"/>
+    <mergeCell ref="B27:B34"/>
     <mergeCell ref="B173"/>
     <mergeCell ref="B63:B67"/>
-    <mergeCell ref="A41:A75"/>
     <mergeCell ref="B104:B106"/>
     <mergeCell ref="B151:B154"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="A142:A154"/>
+    <mergeCell ref="B119:B121"/>
+    <mergeCell ref="A185:A188"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="A155:A156"/>
+    <mergeCell ref="A157:A163"/>
+    <mergeCell ref="A76:A87"/>
+    <mergeCell ref="A41:A75"/>
     <mergeCell ref="A164:A165"/>
     <mergeCell ref="A107:A118"/>
     <mergeCell ref="B36:B40"/>
@@ -5855,20 +5875,6 @@
     <mergeCell ref="B80:B84"/>
     <mergeCell ref="B85:B87"/>
     <mergeCell ref="A89:A103"/>
-    <mergeCell ref="B172"/>
-    <mergeCell ref="A3:A40"/>
-    <mergeCell ref="B76:B79"/>
-    <mergeCell ref="A166:A171"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="B107:B113"/>
-    <mergeCell ref="A172:A184"/>
-    <mergeCell ref="B146:B150"/>
-    <mergeCell ref="B183:B184"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B155:B156"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="B157:B163"/>
-    <mergeCell ref="B136:B137"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5880,18 +5886,18 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -5926,10 +5932,10 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -5954,8 +5960,8 @@
       <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
@@ -5978,8 +5984,8 @@
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -6002,8 +6008,8 @@
       <c r="J5" s="3"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
       <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
@@ -6026,8 +6032,8 @@
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
       <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
@@ -6050,8 +6056,8 @@
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
@@ -6074,8 +6080,8 @@
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
       <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
@@ -6098,8 +6104,8 @@
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
       <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
@@ -6122,8 +6128,8 @@
       <c r="J10" s="3"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
       <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
@@ -6146,8 +6152,8 @@
       <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="6"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -6172,8 +6178,8 @@
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
       <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
@@ -6200,8 +6206,8 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
       <c r="C14" s="3" t="s">
         <v>19</v>
       </c>
@@ -6224,8 +6230,8 @@
       <c r="J14" s="3"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
       <c r="C15" s="3" t="s">
         <v>19</v>
       </c>
@@ -6248,8 +6254,8 @@
       <c r="J15" s="3"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
       <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
@@ -6276,8 +6282,8 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
       <c r="C17" s="3" t="s">
         <v>22</v>
       </c>
@@ -6304,8 +6310,8 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
       <c r="C18" s="3" t="s">
         <v>22</v>
       </c>
@@ -6332,8 +6338,8 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -6358,8 +6364,8 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
       <c r="C20" s="3" t="s">
         <v>22</v>
       </c>
@@ -6382,8 +6388,8 @@
       <c r="J20" s="3"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
       <c r="C21" s="3" t="s">
         <v>22</v>
       </c>
@@ -6406,8 +6412,8 @@
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="9"/>
+      <c r="B22" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -6434,8 +6440,8 @@
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
       <c r="C23" s="3" t="s">
         <v>19</v>
       </c>
@@ -6458,8 +6464,8 @@
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
       <c r="C24" s="3" t="s">
         <v>22</v>
       </c>
@@ -6486,8 +6492,8 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
       <c r="C25" s="3" t="s">
         <v>22</v>
       </c>
@@ -6514,8 +6520,8 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
       <c r="C26" s="3" t="s">
         <v>44</v>
       </c>
@@ -6538,8 +6544,8 @@
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="6"/>
-      <c r="B27" s="7" t="s">
+      <c r="A27" s="9"/>
+      <c r="B27" s="5" t="s">
         <v>46</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -6564,8 +6570,8 @@
       <c r="J27" s="3"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
       <c r="C28" s="3" t="s">
         <v>47</v>
       </c>
@@ -6590,8 +6596,8 @@
       <c r="J28" s="3"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6"/>
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
       <c r="C29" s="3" t="s">
         <v>31</v>
       </c>
@@ -6618,8 +6624,8 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
       <c r="C30" s="3" t="s">
         <v>19</v>
       </c>
@@ -6642,8 +6648,8 @@
       <c r="J30" s="3"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
       <c r="C31" s="3" t="s">
         <v>19</v>
       </c>
@@ -6666,8 +6672,8 @@
       <c r="J31" s="3"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="6"/>
-      <c r="B32" s="6"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
       <c r="C32" s="3" t="s">
         <v>22</v>
       </c>
@@ -6692,8 +6698,8 @@
       <c r="J32" s="3"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
       <c r="C33" s="3" t="s">
         <v>22</v>
       </c>
@@ -6718,8 +6724,8 @@
       <c r="J33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
       <c r="C34" s="3" t="s">
         <v>22</v>
       </c>
@@ -6744,8 +6750,8 @@
       <c r="J34" s="3"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A35" s="6"/>
-      <c r="B35" s="7" t="s">
+      <c r="A35" s="9"/>
+      <c r="B35" s="5" t="s">
         <v>52</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -6772,8 +6778,8 @@
       <c r="J35" s="3"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A36" s="6"/>
-      <c r="B36" s="7" t="s">
+      <c r="A36" s="9"/>
+      <c r="B36" s="5" t="s">
         <v>54</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -6800,8 +6806,8 @@
       <c r="J36" s="3"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" s="6"/>
-      <c r="B37" s="6"/>
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
       <c r="C37" s="3" t="s">
         <v>19</v>
       </c>
@@ -6824,8 +6830,8 @@
       <c r="J37" s="3"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A38" s="6"/>
-      <c r="B38" s="6"/>
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
       <c r="C38" s="3" t="s">
         <v>19</v>
       </c>
@@ -6848,8 +6854,8 @@
       <c r="J38" s="3"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A39" s="6"/>
-      <c r="B39" s="6"/>
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
       <c r="C39" s="3" t="s">
         <v>22</v>
       </c>
@@ -6872,8 +6878,8 @@
       <c r="J39" s="3"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A40" s="6"/>
-      <c r="B40" s="6"/>
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
       <c r="C40" s="3" t="s">
         <v>44</v>
       </c>
@@ -6896,10 +6902,10 @@
       <c r="J40" s="3"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C41" s="4" t="s">
@@ -6926,8 +6932,8 @@
       <c r="J41" s="4"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
+      <c r="A42" s="9"/>
+      <c r="B42" s="9"/>
       <c r="C42" s="4" t="s">
         <v>31</v>
       </c>
@@ -6952,8 +6958,8 @@
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A43" s="6"/>
-      <c r="B43" s="6"/>
+      <c r="A43" s="9"/>
+      <c r="B43" s="9"/>
       <c r="C43" s="4" t="s">
         <v>61</v>
       </c>
@@ -6976,8 +6982,8 @@
       <c r="J43" s="4"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
+      <c r="A44" s="9"/>
+      <c r="B44" s="9"/>
       <c r="C44" s="4" t="s">
         <v>61</v>
       </c>
@@ -7000,8 +7006,8 @@
       <c r="J44" s="4"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A45" s="6"/>
-      <c r="B45" s="6"/>
+      <c r="A45" s="9"/>
+      <c r="B45" s="9"/>
       <c r="C45" s="4" t="s">
         <v>61</v>
       </c>
@@ -7024,8 +7030,8 @@
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A46" s="6"/>
-      <c r="B46" s="6"/>
+      <c r="A46" s="9"/>
+      <c r="B46" s="9"/>
       <c r="C46" s="4" t="s">
         <v>13</v>
       </c>
@@ -7050,8 +7056,8 @@
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
+      <c r="A47" s="9"/>
+      <c r="B47" s="9"/>
       <c r="C47" s="4" t="s">
         <v>13</v>
       </c>
@@ -7076,8 +7082,8 @@
       <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A48" s="6"/>
-      <c r="B48" s="6"/>
+      <c r="A48" s="9"/>
+      <c r="B48" s="9"/>
       <c r="C48" s="4" t="s">
         <v>13</v>
       </c>
@@ -7102,8 +7108,8 @@
       <c r="J48" s="4"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" s="6"/>
-      <c r="B49" s="6"/>
+      <c r="A49" s="9"/>
+      <c r="B49" s="9"/>
       <c r="C49" s="4" t="s">
         <v>19</v>
       </c>
@@ -7126,8 +7132,8 @@
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6"/>
+      <c r="A50" s="9"/>
+      <c r="B50" s="9"/>
       <c r="C50" s="4" t="s">
         <v>19</v>
       </c>
@@ -7150,8 +7156,8 @@
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
+      <c r="A51" s="9"/>
+      <c r="B51" s="9"/>
       <c r="C51" s="4" t="s">
         <v>22</v>
       </c>
@@ -7176,8 +7182,8 @@
       <c r="J51" s="4"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
+      <c r="A52" s="9"/>
+      <c r="B52" s="9"/>
       <c r="C52" s="4" t="s">
         <v>22</v>
       </c>
@@ -7202,8 +7208,8 @@
       <c r="J52" s="4"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
+      <c r="A53" s="9"/>
+      <c r="B53" s="9"/>
       <c r="C53" s="4" t="s">
         <v>22</v>
       </c>
@@ -7228,8 +7234,8 @@
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
+      <c r="A54" s="9"/>
+      <c r="B54" s="9"/>
       <c r="C54" s="4" t="s">
         <v>22</v>
       </c>
@@ -7254,8 +7260,8 @@
       <c r="J54" s="4"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="6"/>
-      <c r="B55" s="5" t="s">
+      <c r="A55" s="9"/>
+      <c r="B55" s="7" t="s">
         <v>64</v>
       </c>
       <c r="C55" s="4" t="s">
@@ -7280,8 +7286,8 @@
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
+      <c r="A56" s="9"/>
+      <c r="B56" s="9"/>
       <c r="C56" s="4" t="s">
         <v>19</v>
       </c>
@@ -7304,8 +7310,8 @@
       <c r="J56" s="4"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
+      <c r="A57" s="9"/>
+      <c r="B57" s="9"/>
       <c r="C57" s="4" t="s">
         <v>22</v>
       </c>
@@ -7328,8 +7334,8 @@
       <c r="J57" s="4"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
+      <c r="A58" s="9"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="4" t="s">
         <v>22</v>
       </c>
@@ -7352,8 +7358,8 @@
       <c r="J58" s="4"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A59" s="6"/>
-      <c r="B59" s="5" t="s">
+      <c r="A59" s="9"/>
+      <c r="B59" s="7" t="s">
         <v>65</v>
       </c>
       <c r="C59" s="4" t="s">
@@ -7380,8 +7386,8 @@
       <c r="J59" s="4"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A60" s="6"/>
-      <c r="B60" s="6"/>
+      <c r="A60" s="9"/>
+      <c r="B60" s="9"/>
       <c r="C60" s="4" t="s">
         <v>22</v>
       </c>
@@ -7406,8 +7412,8 @@
       <c r="J60" s="4"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A61" s="6"/>
-      <c r="B61" s="5" t="s">
+      <c r="A61" s="9"/>
+      <c r="B61" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C61" s="4" t="s">
@@ -7432,8 +7438,8 @@
       <c r="J61" s="4"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="6"/>
-      <c r="B62" s="6"/>
+      <c r="A62" s="9"/>
+      <c r="B62" s="9"/>
       <c r="C62" s="4" t="s">
         <v>22</v>
       </c>
@@ -7458,8 +7464,8 @@
       <c r="J62" s="4"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="6"/>
-      <c r="B63" s="5" t="s">
+      <c r="A63" s="9"/>
+      <c r="B63" s="7" t="s">
         <v>69</v>
       </c>
       <c r="C63" s="4" t="s">
@@ -7488,8 +7494,8 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="6"/>
-      <c r="B64" s="6"/>
+      <c r="A64" s="9"/>
+      <c r="B64" s="9"/>
       <c r="C64" s="4" t="s">
         <v>61</v>
       </c>
@@ -7512,8 +7518,8 @@
       <c r="J64" s="4"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" s="6"/>
-      <c r="B65" s="6"/>
+      <c r="A65" s="9"/>
+      <c r="B65" s="9"/>
       <c r="C65" s="4" t="s">
         <v>19</v>
       </c>
@@ -7536,8 +7542,8 @@
       <c r="J65" s="4"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="6"/>
-      <c r="B66" s="6"/>
+      <c r="A66" s="9"/>
+      <c r="B66" s="9"/>
       <c r="C66" s="4" t="s">
         <v>22</v>
       </c>
@@ -7562,8 +7568,8 @@
       <c r="J66" s="4"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="6"/>
-      <c r="B67" s="6"/>
+      <c r="A67" s="9"/>
+      <c r="B67" s="9"/>
       <c r="C67" s="4" t="s">
         <v>22</v>
       </c>
@@ -7588,8 +7594,8 @@
       <c r="J67" s="4"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A68" s="6"/>
-      <c r="B68" s="5" t="s">
+      <c r="A68" s="9"/>
+      <c r="B68" s="7" t="s">
         <v>71</v>
       </c>
       <c r="C68" s="4" t="s">
@@ -7614,8 +7620,8 @@
       <c r="J68" s="4"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A69" s="6"/>
-      <c r="B69" s="6"/>
+      <c r="A69" s="9"/>
+      <c r="B69" s="9"/>
       <c r="C69" s="4" t="s">
         <v>13</v>
       </c>
@@ -7642,8 +7648,8 @@
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A70" s="6"/>
-      <c r="B70" s="6"/>
+      <c r="A70" s="9"/>
+      <c r="B70" s="9"/>
       <c r="C70" s="4" t="s">
         <v>19</v>
       </c>
@@ -7666,8 +7672,8 @@
       <c r="J70" s="4"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A71" s="6"/>
-      <c r="B71" s="6"/>
+      <c r="A71" s="9"/>
+      <c r="B71" s="9"/>
       <c r="C71" s="4" t="s">
         <v>19</v>
       </c>
@@ -7690,8 +7696,8 @@
       <c r="J71" s="4"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A72" s="6"/>
-      <c r="B72" s="6"/>
+      <c r="A72" s="9"/>
+      <c r="B72" s="9"/>
       <c r="C72" s="4" t="s">
         <v>22</v>
       </c>
@@ -7718,8 +7724,8 @@
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A73" s="6"/>
-      <c r="B73" s="6"/>
+      <c r="A73" s="9"/>
+      <c r="B73" s="9"/>
       <c r="C73" s="4" t="s">
         <v>22</v>
       </c>
@@ -7746,8 +7752,8 @@
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A74" s="6"/>
-      <c r="B74" s="6"/>
+      <c r="A74" s="9"/>
+      <c r="B74" s="9"/>
       <c r="C74" s="4" t="s">
         <v>22</v>
       </c>
@@ -7774,8 +7780,8 @@
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A75" s="6"/>
-      <c r="B75" s="6"/>
+      <c r="A75" s="9"/>
+      <c r="B75" s="9"/>
       <c r="C75" s="4" t="s">
         <v>22</v>
       </c>
@@ -7802,10 +7808,10 @@
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B76" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C76" s="3" t="s">
@@ -7830,8 +7836,8 @@
       <c r="J76" s="3"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A77" s="6"/>
-      <c r="B77" s="6"/>
+      <c r="A77" s="9"/>
+      <c r="B77" s="9"/>
       <c r="C77" s="3" t="s">
         <v>19</v>
       </c>
@@ -7854,8 +7860,8 @@
       <c r="J77" s="3"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A78" s="6"/>
-      <c r="B78" s="6"/>
+      <c r="A78" s="9"/>
+      <c r="B78" s="9"/>
       <c r="C78" s="3" t="s">
         <v>19</v>
       </c>
@@ -7878,8 +7884,8 @@
       <c r="J78" s="3"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A79" s="6"/>
-      <c r="B79" s="6"/>
+      <c r="A79" s="9"/>
+      <c r="B79" s="9"/>
       <c r="C79" s="3" t="s">
         <v>22</v>
       </c>
@@ -7902,8 +7908,8 @@
       <c r="J79" s="3"/>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A80" s="6"/>
-      <c r="B80" s="7" t="s">
+      <c r="A80" s="9"/>
+      <c r="B80" s="5" t="s">
         <v>77</v>
       </c>
       <c r="C80" s="3" t="s">
@@ -7930,8 +7936,8 @@
       <c r="J80" s="3"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A81" s="6"/>
-      <c r="B81" s="6"/>
+      <c r="A81" s="9"/>
+      <c r="B81" s="9"/>
       <c r="C81" s="3" t="s">
         <v>79</v>
       </c>
@@ -7954,8 +7960,8 @@
       <c r="J81" s="3"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A82" s="6"/>
-      <c r="B82" s="6"/>
+      <c r="A82" s="9"/>
+      <c r="B82" s="9"/>
       <c r="C82" s="3" t="s">
         <v>19</v>
       </c>
@@ -7978,8 +7984,8 @@
       <c r="J82" s="3"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A83" s="6"/>
-      <c r="B83" s="6"/>
+      <c r="A83" s="9"/>
+      <c r="B83" s="9"/>
       <c r="C83" s="3" t="s">
         <v>22</v>
       </c>
@@ -8004,8 +8010,8 @@
       <c r="J83" s="3"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A84" s="6"/>
-      <c r="B84" s="6"/>
+      <c r="A84" s="9"/>
+      <c r="B84" s="9"/>
       <c r="C84" s="3" t="s">
         <v>22</v>
       </c>
@@ -8030,8 +8036,8 @@
       <c r="J84" s="3"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A85" s="6"/>
-      <c r="B85" s="7" t="s">
+      <c r="A85" s="9"/>
+      <c r="B85" s="5" t="s">
         <v>81</v>
       </c>
       <c r="C85" s="3" t="s">
@@ -8056,8 +8062,8 @@
       <c r="J85" s="3"/>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A86" s="6"/>
-      <c r="B86" s="6"/>
+      <c r="A86" s="9"/>
+      <c r="B86" s="9"/>
       <c r="C86" s="3" t="s">
         <v>19</v>
       </c>
@@ -8080,8 +8086,8 @@
       <c r="J86" s="3"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A87" s="6"/>
-      <c r="B87" s="6"/>
+      <c r="A87" s="9"/>
+      <c r="B87" s="9"/>
       <c r="C87" s="3" t="s">
         <v>22</v>
       </c>
@@ -8107,7 +8113,7 @@
       <c r="A88" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="7" t="s">
         <v>83</v>
       </c>
       <c r="C88" s="4" t="s">
@@ -8136,10 +8142,10 @@
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A89" s="8" t="s">
+      <c r="A89" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="B89" s="5" t="s">
         <v>87</v>
       </c>
       <c r="C89" s="3" t="s">
@@ -8166,8 +8172,8 @@
       <c r="J89" s="3"/>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A90" s="6"/>
-      <c r="B90" s="6"/>
+      <c r="A90" s="9"/>
+      <c r="B90" s="9"/>
       <c r="C90" s="3" t="s">
         <v>19</v>
       </c>
@@ -8190,8 +8196,8 @@
       <c r="J90" s="3"/>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A91" s="6"/>
-      <c r="B91" s="6"/>
+      <c r="A91" s="9"/>
+      <c r="B91" s="9"/>
       <c r="C91" s="3" t="s">
         <v>19</v>
       </c>
@@ -8214,8 +8220,8 @@
       <c r="J91" s="3"/>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A92" s="6"/>
-      <c r="B92" s="6"/>
+      <c r="A92" s="9"/>
+      <c r="B92" s="9"/>
       <c r="C92" s="3" t="s">
         <v>22</v>
       </c>
@@ -8240,8 +8246,8 @@
       <c r="J92" s="3"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A93" s="6"/>
-      <c r="B93" s="7" t="s">
+      <c r="A93" s="9"/>
+      <c r="B93" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C93" s="3" t="s">
@@ -8268,8 +8274,8 @@
       <c r="J93" s="3"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A94" s="6"/>
-      <c r="B94" s="6"/>
+      <c r="A94" s="9"/>
+      <c r="B94" s="9"/>
       <c r="C94" s="3" t="s">
         <v>19</v>
       </c>
@@ -8292,8 +8298,8 @@
       <c r="J94" s="3"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A95" s="6"/>
-      <c r="B95" s="6"/>
+      <c r="A95" s="9"/>
+      <c r="B95" s="9"/>
       <c r="C95" s="3" t="s">
         <v>22</v>
       </c>
@@ -8318,8 +8324,8 @@
       <c r="J95" s="3"/>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A96" s="6"/>
-      <c r="B96" s="6"/>
+      <c r="A96" s="9"/>
+      <c r="B96" s="9"/>
       <c r="C96" s="3" t="s">
         <v>22</v>
       </c>
@@ -8344,8 +8350,8 @@
       <c r="J96" s="3"/>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A97" s="6"/>
-      <c r="B97" s="6"/>
+      <c r="A97" s="9"/>
+      <c r="B97" s="9"/>
       <c r="C97" s="3" t="s">
         <v>22</v>
       </c>
@@ -8370,8 +8376,8 @@
       <c r="J97" s="3"/>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A98" s="6"/>
-      <c r="B98" s="7" t="s">
+      <c r="A98" s="9"/>
+      <c r="B98" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C98" s="3" t="s">
@@ -8398,8 +8404,8 @@
       <c r="J98" s="3"/>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6"/>
+      <c r="A99" s="9"/>
+      <c r="B99" s="9"/>
       <c r="C99" s="3" t="s">
         <v>61</v>
       </c>
@@ -8422,8 +8428,8 @@
       <c r="J99" s="3"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A100" s="6"/>
-      <c r="B100" s="6"/>
+      <c r="A100" s="9"/>
+      <c r="B100" s="9"/>
       <c r="C100" s="3" t="s">
         <v>22</v>
       </c>
@@ -8448,8 +8454,8 @@
       <c r="J100" s="3"/>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A101" s="6"/>
-      <c r="B101" s="7" t="s">
+      <c r="A101" s="9"/>
+      <c r="B101" s="5" t="s">
         <v>93</v>
       </c>
       <c r="C101" s="3" t="s">
@@ -8476,8 +8482,8 @@
       <c r="J101" s="3"/>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6"/>
+      <c r="A102" s="9"/>
+      <c r="B102" s="9"/>
       <c r="C102" s="3" t="s">
         <v>95</v>
       </c>
@@ -8496,8 +8502,8 @@
       <c r="J102" s="3"/>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A103" s="6"/>
-      <c r="B103" s="6"/>
+      <c r="A103" s="9"/>
+      <c r="B103" s="9"/>
       <c r="C103" s="3" t="s">
         <v>95</v>
       </c>
@@ -8516,10 +8522,10 @@
       <c r="J103" s="3"/>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A104" s="8" t="s">
+      <c r="A104" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B104" s="7" t="s">
         <v>98</v>
       </c>
       <c r="C104" s="4" t="s">
@@ -8546,8 +8552,8 @@
       <c r="J104" s="4"/>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6"/>
+      <c r="A105" s="9"/>
+      <c r="B105" s="9"/>
       <c r="C105" s="4" t="s">
         <v>61</v>
       </c>
@@ -8570,8 +8576,8 @@
       <c r="J105" s="4"/>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A106" s="6"/>
-      <c r="B106" s="6"/>
+      <c r="A106" s="9"/>
+      <c r="B106" s="9"/>
       <c r="C106" s="4" t="s">
         <v>100</v>
       </c>
@@ -8596,10 +8602,10 @@
       <c r="J106" s="4"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A107" s="8" t="s">
+      <c r="A107" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B107" s="7" t="s">
+      <c r="B107" s="5" t="s">
         <v>103</v>
       </c>
       <c r="C107" s="3" t="s">
@@ -8626,8 +8632,8 @@
       <c r="J107" s="3"/>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A108" s="6"/>
-      <c r="B108" s="6"/>
+      <c r="A108" s="9"/>
+      <c r="B108" s="9"/>
       <c r="C108" s="3" t="s">
         <v>47</v>
       </c>
@@ -8652,8 +8658,8 @@
       <c r="J108" s="3"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A109" s="6"/>
-      <c r="B109" s="6"/>
+      <c r="A109" s="9"/>
+      <c r="B109" s="9"/>
       <c r="C109" s="3" t="s">
         <v>61</v>
       </c>
@@ -8676,8 +8682,8 @@
       <c r="J109" s="3"/>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A110" s="6"/>
-      <c r="B110" s="6"/>
+      <c r="A110" s="9"/>
+      <c r="B110" s="9"/>
       <c r="C110" s="3" t="s">
         <v>19</v>
       </c>
@@ -8700,8 +8706,8 @@
       <c r="J110" s="3"/>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A111" s="6"/>
-      <c r="B111" s="6"/>
+      <c r="A111" s="9"/>
+      <c r="B111" s="9"/>
       <c r="C111" s="3" t="s">
         <v>22</v>
       </c>
@@ -8726,8 +8732,8 @@
       <c r="J111" s="3"/>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A112" s="6"/>
-      <c r="B112" s="6"/>
+      <c r="A112" s="9"/>
+      <c r="B112" s="9"/>
       <c r="C112" s="3" t="s">
         <v>22</v>
       </c>
@@ -8752,8 +8758,8 @@
       <c r="J112" s="3"/>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A113" s="6"/>
-      <c r="B113" s="6"/>
+      <c r="A113" s="9"/>
+      <c r="B113" s="9"/>
       <c r="C113" s="3" t="s">
         <v>22</v>
       </c>
@@ -8778,8 +8784,8 @@
       <c r="J113" s="3"/>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A114" s="6"/>
-      <c r="B114" s="7" t="s">
+      <c r="A114" s="9"/>
+      <c r="B114" s="5" t="s">
         <v>105</v>
       </c>
       <c r="C114" s="3" t="s">
@@ -8804,8 +8810,8 @@
       <c r="J114" s="3"/>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A115" s="6"/>
-      <c r="B115" s="6"/>
+      <c r="A115" s="9"/>
+      <c r="B115" s="9"/>
       <c r="C115" s="3" t="s">
         <v>22</v>
       </c>
@@ -8830,8 +8836,8 @@
       <c r="J115" s="3"/>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A116" s="6"/>
-      <c r="B116" s="7" t="s">
+      <c r="A116" s="9"/>
+      <c r="B116" s="5" t="s">
         <v>107</v>
       </c>
       <c r="C116" s="3" t="s">
@@ -8858,8 +8864,8 @@
       <c r="J116" s="3"/>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A117" s="6"/>
-      <c r="B117" s="6"/>
+      <c r="A117" s="9"/>
+      <c r="B117" s="9"/>
       <c r="C117" s="3" t="s">
         <v>19</v>
       </c>
@@ -8882,8 +8888,8 @@
       <c r="J117" s="3"/>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A118" s="6"/>
-      <c r="B118" s="6"/>
+      <c r="A118" s="9"/>
+      <c r="B118" s="9"/>
       <c r="C118" s="3" t="s">
         <v>22</v>
       </c>
@@ -8910,10 +8916,10 @@
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A119" s="8" t="s">
+      <c r="A119" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B119" s="5" t="s">
+      <c r="B119" s="7" t="s">
         <v>111</v>
       </c>
       <c r="C119" s="4" t="s">
@@ -8938,8 +8944,8 @@
       <c r="J119" s="4"/>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A120" s="6"/>
-      <c r="B120" s="6"/>
+      <c r="A120" s="9"/>
+      <c r="B120" s="9"/>
       <c r="C120" s="4" t="s">
         <v>112</v>
       </c>
@@ -8962,8 +8968,8 @@
       <c r="J120" s="4"/>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A121" s="6"/>
-      <c r="B121" s="6"/>
+      <c r="A121" s="9"/>
+      <c r="B121" s="9"/>
       <c r="C121" s="4" t="s">
         <v>112</v>
       </c>
@@ -8986,8 +8992,8 @@
       <c r="J121" s="4"/>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A122" s="6"/>
-      <c r="B122" s="5" t="s">
+      <c r="A122" s="9"/>
+      <c r="B122" s="7" t="s">
         <v>114</v>
       </c>
       <c r="C122" s="4" t="s">
@@ -9016,8 +9022,8 @@
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A123" s="6"/>
-      <c r="B123" s="6"/>
+      <c r="A123" s="9"/>
+      <c r="B123" s="9"/>
       <c r="C123" s="4" t="s">
         <v>61</v>
       </c>
@@ -9040,8 +9046,8 @@
       <c r="J123" s="4"/>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A124" s="6"/>
-      <c r="B124" s="6"/>
+      <c r="A124" s="9"/>
+      <c r="B124" s="9"/>
       <c r="C124" s="4" t="s">
         <v>112</v>
       </c>
@@ -9066,8 +9072,8 @@
       <c r="J124" s="4"/>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A125" s="6"/>
-      <c r="B125" s="6"/>
+      <c r="A125" s="9"/>
+      <c r="B125" s="9"/>
       <c r="C125" s="4" t="s">
         <v>112</v>
       </c>
@@ -9092,8 +9098,8 @@
       <c r="J125" s="4"/>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A126" s="6"/>
-      <c r="B126" s="5" t="s">
+      <c r="A126" s="9"/>
+      <c r="B126" s="7" t="s">
         <v>118</v>
       </c>
       <c r="C126" s="4" t="s">
@@ -9118,8 +9124,8 @@
       <c r="J126" s="4"/>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A127" s="6"/>
-      <c r="B127" s="6"/>
+      <c r="A127" s="9"/>
+      <c r="B127" s="9"/>
       <c r="C127" s="4" t="s">
         <v>112</v>
       </c>
@@ -9142,8 +9148,8 @@
       <c r="J127" s="4"/>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A128" s="6"/>
-      <c r="B128" s="5" t="s">
+      <c r="A128" s="9"/>
+      <c r="B128" s="7" t="s">
         <v>119</v>
       </c>
       <c r="C128" s="4" t="s">
@@ -9170,8 +9176,8 @@
       <c r="J128" s="4"/>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A129" s="6"/>
-      <c r="B129" s="6"/>
+      <c r="A129" s="9"/>
+      <c r="B129" s="9"/>
       <c r="C129" s="4" t="s">
         <v>100</v>
       </c>
@@ -9196,8 +9202,8 @@
       <c r="J129" s="4"/>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A130" s="6"/>
-      <c r="B130" s="6"/>
+      <c r="A130" s="9"/>
+      <c r="B130" s="9"/>
       <c r="C130" s="4" t="s">
         <v>112</v>
       </c>
@@ -9220,8 +9226,8 @@
       <c r="J130" s="4"/>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A131" s="6"/>
-      <c r="B131" s="5" t="s">
+      <c r="A131" s="9"/>
+      <c r="B131" s="7" t="s">
         <v>121</v>
       </c>
       <c r="C131" s="4" t="s">
@@ -9250,8 +9256,8 @@
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A132" s="6"/>
-      <c r="B132" s="6"/>
+      <c r="A132" s="9"/>
+      <c r="B132" s="9"/>
       <c r="C132" s="4" t="s">
         <v>100</v>
       </c>
@@ -9278,8 +9284,8 @@
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A133" s="6"/>
-      <c r="B133" s="6"/>
+      <c r="A133" s="9"/>
+      <c r="B133" s="9"/>
       <c r="C133" s="4" t="s">
         <v>112</v>
       </c>
@@ -9306,8 +9312,8 @@
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A134" s="6"/>
-      <c r="B134" s="6"/>
+      <c r="A134" s="9"/>
+      <c r="B134" s="9"/>
       <c r="C134" s="4" t="s">
         <v>112</v>
       </c>
@@ -9334,8 +9340,8 @@
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A135" s="6"/>
-      <c r="B135" s="6"/>
+      <c r="A135" s="9"/>
+      <c r="B135" s="9"/>
       <c r="C135" s="4" t="s">
         <v>112</v>
       </c>
@@ -9362,8 +9368,8 @@
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A136" s="6"/>
-      <c r="B136" s="5" t="s">
+      <c r="A136" s="9"/>
+      <c r="B136" s="7" t="s">
         <v>124</v>
       </c>
       <c r="C136" s="4" t="s">
@@ -9390,8 +9396,8 @@
       <c r="J136" s="4"/>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A137" s="6"/>
-      <c r="B137" s="6"/>
+      <c r="A137" s="9"/>
+      <c r="B137" s="9"/>
       <c r="C137" s="4" t="s">
         <v>112</v>
       </c>
@@ -9416,8 +9422,8 @@
       <c r="J137" s="4"/>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A138" s="6"/>
-      <c r="B138" s="5" t="s">
+      <c r="A138" s="9"/>
+      <c r="B138" s="7" t="s">
         <v>126</v>
       </c>
       <c r="C138" s="4" t="s">
@@ -9442,8 +9448,8 @@
       <c r="J138" s="4"/>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A139" s="6"/>
-      <c r="B139" s="6"/>
+      <c r="A139" s="9"/>
+      <c r="B139" s="9"/>
       <c r="C139" s="4" t="s">
         <v>112</v>
       </c>
@@ -9466,8 +9472,8 @@
       <c r="J139" s="4"/>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A140" s="6"/>
-      <c r="B140" s="6"/>
+      <c r="A140" s="9"/>
+      <c r="B140" s="9"/>
       <c r="C140" s="4" t="s">
         <v>112</v>
       </c>
@@ -9490,8 +9496,8 @@
       <c r="J140" s="4"/>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A141" s="6"/>
-      <c r="B141" s="6"/>
+      <c r="A141" s="9"/>
+      <c r="B141" s="9"/>
       <c r="C141" s="4" t="s">
         <v>112</v>
       </c>
@@ -9514,10 +9520,10 @@
       <c r="J141" s="4"/>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A142" s="8" t="s">
+      <c r="A142" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B142" s="7" t="s">
+      <c r="B142" s="5" t="s">
         <v>128</v>
       </c>
       <c r="C142" s="3" t="s">
@@ -9544,8 +9550,8 @@
       <c r="J142" s="3"/>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A143" s="6"/>
-      <c r="B143" s="6"/>
+      <c r="A143" s="9"/>
+      <c r="B143" s="9"/>
       <c r="C143" s="3" t="s">
         <v>100</v>
       </c>
@@ -9570,8 +9576,8 @@
       <c r="J143" s="3"/>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
+      <c r="A144" s="9"/>
+      <c r="B144" s="9"/>
       <c r="C144" s="3" t="s">
         <v>112</v>
       </c>
@@ -9596,8 +9602,8 @@
       <c r="J144" s="3"/>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A145" s="6"/>
-      <c r="B145" s="6"/>
+      <c r="A145" s="9"/>
+      <c r="B145" s="9"/>
       <c r="C145" s="3" t="s">
         <v>112</v>
       </c>
@@ -9622,8 +9628,8 @@
       <c r="J145" s="3"/>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A146" s="6"/>
-      <c r="B146" s="7" t="s">
+      <c r="A146" s="9"/>
+      <c r="B146" s="5" t="s">
         <v>130</v>
       </c>
       <c r="C146" s="3" t="s">
@@ -9650,8 +9656,8 @@
       <c r="J146" s="3"/>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A147" s="6"/>
-      <c r="B147" s="6"/>
+      <c r="A147" s="9"/>
+      <c r="B147" s="9"/>
       <c r="C147" s="3" t="s">
         <v>61</v>
       </c>
@@ -9674,8 +9680,8 @@
       <c r="J147" s="3"/>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A148" s="6"/>
-      <c r="B148" s="6"/>
+      <c r="A148" s="9"/>
+      <c r="B148" s="9"/>
       <c r="C148" s="3" t="s">
         <v>100</v>
       </c>
@@ -9700,8 +9706,8 @@
       <c r="J148" s="3"/>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A149" s="6"/>
-      <c r="B149" s="6"/>
+      <c r="A149" s="9"/>
+      <c r="B149" s="9"/>
       <c r="C149" s="3" t="s">
         <v>112</v>
       </c>
@@ -9726,8 +9732,8 @@
       <c r="J149" s="3"/>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A150" s="6"/>
-      <c r="B150" s="6"/>
+      <c r="A150" s="9"/>
+      <c r="B150" s="9"/>
       <c r="C150" s="3" t="s">
         <v>112</v>
       </c>
@@ -9752,8 +9758,8 @@
       <c r="J150" s="3"/>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A151" s="6"/>
-      <c r="B151" s="7" t="s">
+      <c r="A151" s="9"/>
+      <c r="B151" s="5" t="s">
         <v>135</v>
       </c>
       <c r="C151" s="3" t="s">
@@ -9780,8 +9786,8 @@
       <c r="J151" s="3"/>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A152" s="6"/>
-      <c r="B152" s="6"/>
+      <c r="A152" s="9"/>
+      <c r="B152" s="9"/>
       <c r="C152" s="3" t="s">
         <v>100</v>
       </c>
@@ -9806,8 +9812,8 @@
       <c r="J152" s="3"/>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A153" s="6"/>
-      <c r="B153" s="6"/>
+      <c r="A153" s="9"/>
+      <c r="B153" s="9"/>
       <c r="C153" s="3" t="s">
         <v>112</v>
       </c>
@@ -9832,8 +9838,8 @@
       <c r="J153" s="3"/>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A154" s="6"/>
-      <c r="B154" s="6"/>
+      <c r="A154" s="9"/>
+      <c r="B154" s="9"/>
       <c r="C154" s="3" t="s">
         <v>112</v>
       </c>
@@ -9858,10 +9864,10 @@
       <c r="J154" s="3"/>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A155" s="8" t="s">
+      <c r="A155" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B155" s="5" t="s">
+      <c r="B155" s="7" t="s">
         <v>138</v>
       </c>
       <c r="C155" s="4" t="s">
@@ -9886,8 +9892,8 @@
       <c r="J155" s="4"/>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A156" s="6"/>
-      <c r="B156" s="6"/>
+      <c r="A156" s="9"/>
+      <c r="B156" s="9"/>
       <c r="C156" s="4" t="s">
         <v>112</v>
       </c>
@@ -9912,10 +9918,10 @@
       <c r="J156" s="4"/>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A157" s="8" t="s">
+      <c r="A157" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B157" s="7" t="s">
+      <c r="B157" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C157" s="3" t="s">
@@ -9942,8 +9948,8 @@
       <c r="J157" s="3"/>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A158" s="6"/>
-      <c r="B158" s="6"/>
+      <c r="A158" s="9"/>
+      <c r="B158" s="9"/>
       <c r="C158" s="3" t="s">
         <v>115</v>
       </c>
@@ -9970,8 +9976,8 @@
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A159" s="6"/>
-      <c r="B159" s="6"/>
+      <c r="A159" s="9"/>
+      <c r="B159" s="9"/>
       <c r="C159" s="3" t="s">
         <v>100</v>
       </c>
@@ -9996,8 +10002,8 @@
       <c r="J159" s="3"/>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A160" s="6"/>
-      <c r="B160" s="6"/>
+      <c r="A160" s="9"/>
+      <c r="B160" s="9"/>
       <c r="C160" s="3" t="s">
         <v>112</v>
       </c>
@@ -10020,8 +10026,8 @@
       <c r="J160" s="3"/>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A161" s="6"/>
-      <c r="B161" s="6"/>
+      <c r="A161" s="9"/>
+      <c r="B161" s="9"/>
       <c r="C161" s="3" t="s">
         <v>112</v>
       </c>
@@ -10044,8 +10050,8 @@
       <c r="J161" s="3"/>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A162" s="6"/>
-      <c r="B162" s="6"/>
+      <c r="A162" s="9"/>
+      <c r="B162" s="9"/>
       <c r="C162" s="3" t="s">
         <v>112</v>
       </c>
@@ -10068,8 +10074,8 @@
       <c r="J162" s="3"/>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A163" s="6"/>
-      <c r="B163" s="6"/>
+      <c r="A163" s="9"/>
+      <c r="B163" s="9"/>
       <c r="C163" s="3" t="s">
         <v>44</v>
       </c>
@@ -10092,10 +10098,10 @@
       <c r="J163" s="3"/>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A164" s="8" t="s">
+      <c r="A164" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B164" s="5" t="s">
+      <c r="B164" s="7" t="s">
         <v>147</v>
       </c>
       <c r="C164" s="4" t="s">
@@ -10122,8 +10128,8 @@
       <c r="J164" s="4"/>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A165" s="6"/>
-      <c r="B165" s="6"/>
+      <c r="A165" s="9"/>
+      <c r="B165" s="9"/>
       <c r="C165" s="4" t="s">
         <v>112</v>
       </c>
@@ -10148,10 +10154,10 @@
       <c r="J165" s="4"/>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A166" s="8" t="s">
+      <c r="A166" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B166" s="7" t="s">
+      <c r="B166" s="5" t="s">
         <v>150</v>
       </c>
       <c r="C166" s="3" t="s">
@@ -10178,8 +10184,8 @@
       <c r="J166" s="3"/>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A167" s="6"/>
-      <c r="B167" s="6"/>
+      <c r="A167" s="9"/>
+      <c r="B167" s="9"/>
       <c r="C167" s="3" t="s">
         <v>112</v>
       </c>
@@ -10204,8 +10210,8 @@
       <c r="J167" s="3"/>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A168" s="6"/>
-      <c r="B168" s="6"/>
+      <c r="A168" s="9"/>
+      <c r="B168" s="9"/>
       <c r="C168" s="3" t="s">
         <v>112</v>
       </c>
@@ -10230,8 +10236,8 @@
       <c r="J168" s="3"/>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A169" s="6"/>
-      <c r="B169" s="7" t="s">
+      <c r="A169" s="9"/>
+      <c r="B169" s="5" t="s">
         <v>152</v>
       </c>
       <c r="C169" s="3" t="s">
@@ -10258,8 +10264,8 @@
       <c r="J169" s="3"/>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A170" s="6"/>
-      <c r="B170" s="6"/>
+      <c r="A170" s="9"/>
+      <c r="B170" s="9"/>
       <c r="C170" s="3" t="s">
         <v>112</v>
       </c>
@@ -10284,8 +10290,8 @@
       <c r="J170" s="3"/>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A171" s="6"/>
-      <c r="B171" s="7" t="s">
+      <c r="A171" s="9"/>
+      <c r="B171" s="5" t="s">
         <v>156</v>
       </c>
       <c r="C171" s="3" t="s">
@@ -10310,10 +10316,10 @@
       <c r="J171" s="3"/>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A172" s="8" t="s">
+      <c r="A172" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B172" s="5" t="s">
+      <c r="B172" s="7" t="s">
         <v>158</v>
       </c>
       <c r="C172" s="4" t="s">
@@ -10340,8 +10346,8 @@
       <c r="J172" s="4"/>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A173" s="6"/>
-      <c r="B173" s="5" t="s">
+      <c r="A173" s="9"/>
+      <c r="B173" s="7" t="s">
         <v>160</v>
       </c>
       <c r="C173" s="4" t="s">
@@ -10368,8 +10374,8 @@
       <c r="J173" s="4"/>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A174" s="6"/>
-      <c r="B174" s="5" t="s">
+      <c r="A174" s="9"/>
+      <c r="B174" s="7" t="s">
         <v>162</v>
       </c>
       <c r="C174" s="4" t="s">
@@ -10394,8 +10400,8 @@
       <c r="J174" s="4"/>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A175" s="6"/>
-      <c r="B175" s="6"/>
+      <c r="A175" s="9"/>
+      <c r="B175" s="9"/>
       <c r="C175" s="4" t="s">
         <v>163</v>
       </c>
@@ -10418,8 +10424,8 @@
       <c r="J175" s="4"/>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A176" s="6"/>
-      <c r="B176" s="6"/>
+      <c r="A176" s="9"/>
+      <c r="B176" s="9"/>
       <c r="C176" s="4" t="s">
         <v>95</v>
       </c>
@@ -10438,8 +10444,8 @@
       <c r="J176" s="4"/>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A177" s="6"/>
-      <c r="B177" s="6"/>
+      <c r="A177" s="9"/>
+      <c r="B177" s="9"/>
       <c r="C177" s="4" t="s">
         <v>112</v>
       </c>
@@ -10464,8 +10470,8 @@
       <c r="J177" s="4"/>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A178" s="6"/>
-      <c r="B178" s="6"/>
+      <c r="A178" s="9"/>
+      <c r="B178" s="9"/>
       <c r="C178" s="4" t="s">
         <v>112</v>
       </c>
@@ -10490,8 +10496,8 @@
       <c r="J178" s="4"/>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A179" s="6"/>
-      <c r="B179" s="6"/>
+      <c r="A179" s="9"/>
+      <c r="B179" s="9"/>
       <c r="C179" s="4" t="s">
         <v>112</v>
       </c>
@@ -10516,8 +10522,8 @@
       <c r="J179" s="4"/>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A180" s="6"/>
-      <c r="B180" s="5" t="s">
+      <c r="A180" s="9"/>
+      <c r="B180" s="7" t="s">
         <v>166</v>
       </c>
       <c r="C180" s="4" t="s">
@@ -10542,8 +10548,8 @@
       <c r="J180" s="4"/>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A181" s="6"/>
-      <c r="B181" s="6"/>
+      <c r="A181" s="9"/>
+      <c r="B181" s="9"/>
       <c r="C181" s="4" t="s">
         <v>163</v>
       </c>
@@ -10566,8 +10572,8 @@
       <c r="J181" s="4"/>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A182" s="6"/>
-      <c r="B182" s="6"/>
+      <c r="A182" s="9"/>
+      <c r="B182" s="9"/>
       <c r="C182" s="4" t="s">
         <v>112</v>
       </c>
@@ -10590,8 +10596,8 @@
       <c r="J182" s="4"/>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A183" s="6"/>
-      <c r="B183" s="5" t="s">
+      <c r="A183" s="9"/>
+      <c r="B183" s="7" t="s">
         <v>167</v>
       </c>
       <c r="C183" s="4" t="s">
@@ -10620,8 +10626,8 @@
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A184" s="6"/>
-      <c r="B184" s="6"/>
+      <c r="A184" s="9"/>
+      <c r="B184" s="9"/>
       <c r="C184" s="4" t="s">
         <v>112</v>
       </c>
@@ -10648,10 +10654,10 @@
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A185" s="8" t="s">
+      <c r="A185" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B185" s="7" t="s">
+      <c r="B185" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C185" s="3" t="s">
@@ -10678,8 +10684,8 @@
       <c r="J185" s="3"/>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A186" s="6"/>
-      <c r="B186" s="6"/>
+      <c r="A186" s="9"/>
+      <c r="B186" s="9"/>
       <c r="C186" s="3" t="s">
         <v>100</v>
       </c>
@@ -10704,8 +10710,8 @@
       <c r="J186" s="3"/>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A187" s="6"/>
-      <c r="B187" s="6"/>
+      <c r="A187" s="9"/>
+      <c r="B187" s="9"/>
       <c r="C187" s="3" t="s">
         <v>112</v>
       </c>
@@ -10728,8 +10734,8 @@
       <c r="J187" s="3"/>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A188" s="6"/>
-      <c r="B188" s="6"/>
+      <c r="A188" s="9"/>
+      <c r="B188" s="9"/>
       <c r="C188" s="3" t="s">
         <v>112</v>
       </c>
@@ -10753,26 +10759,20 @@
     </row>
   </sheetData>
   <mergeCells count="62">
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="B119:B121"/>
-    <mergeCell ref="A142:A154"/>
-    <mergeCell ref="A185:A188"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B12:B18"/>
-    <mergeCell ref="B164:B165"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="B185:B188"/>
-    <mergeCell ref="B93:B97"/>
-    <mergeCell ref="B101:B103"/>
-    <mergeCell ref="A155:A156"/>
-    <mergeCell ref="B114:B115"/>
-    <mergeCell ref="B116:B118"/>
-    <mergeCell ref="A157:A163"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="A76:A87"/>
-    <mergeCell ref="B88"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="B27:B34"/>
+    <mergeCell ref="A172:A184"/>
+    <mergeCell ref="B146:B150"/>
+    <mergeCell ref="B183:B184"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="B157:B163"/>
+    <mergeCell ref="B136:B137"/>
+    <mergeCell ref="A3:A40"/>
+    <mergeCell ref="B76:B79"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="A166:A171"/>
+    <mergeCell ref="B61:B62"/>
+    <mergeCell ref="B107:B113"/>
+    <mergeCell ref="B122:B125"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A119:A141"/>
     <mergeCell ref="B131:B135"/>
@@ -10789,11 +10789,31 @@
     <mergeCell ref="B138:B141"/>
     <mergeCell ref="B172"/>
     <mergeCell ref="B35"/>
+    <mergeCell ref="B12:B18"/>
+    <mergeCell ref="B164:B165"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="B185:B188"/>
+    <mergeCell ref="B93:B97"/>
+    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="B116:B118"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="B88"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="B27:B34"/>
     <mergeCell ref="B173"/>
     <mergeCell ref="B63:B67"/>
-    <mergeCell ref="A41:A75"/>
     <mergeCell ref="B104:B106"/>
     <mergeCell ref="B151:B154"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="B119:B121"/>
+    <mergeCell ref="A142:A154"/>
+    <mergeCell ref="A185:A188"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="A155:A156"/>
+    <mergeCell ref="A157:A163"/>
+    <mergeCell ref="A76:A87"/>
+    <mergeCell ref="A41:A75"/>
     <mergeCell ref="A164:A165"/>
     <mergeCell ref="A107:A118"/>
     <mergeCell ref="B36:B40"/>
@@ -10801,20 +10821,6 @@
     <mergeCell ref="B80:B84"/>
     <mergeCell ref="B85:B87"/>
     <mergeCell ref="A89:A103"/>
-    <mergeCell ref="A3:A40"/>
-    <mergeCell ref="B76:B79"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="A166:A171"/>
-    <mergeCell ref="B61:B62"/>
-    <mergeCell ref="B107:B113"/>
-    <mergeCell ref="A172:A184"/>
-    <mergeCell ref="B146:B150"/>
-    <mergeCell ref="B183:B184"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B155:B156"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="B157:B163"/>
-    <mergeCell ref="B136:B137"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>